<commit_message>
Checkin 3 for Render hosting
</commit_message>
<xml_diff>
--- a/JobAutoApplyMvc/JobAutoApply.Web/Data/JobApplications.xlsx
+++ b/JobAutoApplyMvc/JobAutoApply.Web/Data/JobApplications.xlsx
@@ -81,6 +81,54 @@
   <x:si>
     <x:t>https://www.naukri.com/job-listings-full-stack-net-developer-capgemini-pune-6-to-10-years-190526015463</x:t>
   </x:si>
+  <x:si>
+    <x:t>https://www.naukri.com/job-listings-software-engineer-net-developer-cgi-information-systems-and-management-consultants-hyderabad-1-to-4-years-130526503452</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Apply on company site</x:t>
+  </x:si>
+  <x:si>
+    <x:t>External apply required</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Saved for manual apply on company website.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.naukri.com/job-listings-net-developer-webforms-injala-ahmedabad-2-to-3-years-210126025809</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Apply attempt</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Clicked not confirmed</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Apply was clicked, but no applied confirmation was detected.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.naukri.com/job-listings-dot-net-developer-lion-vision-technology-ahmedabad-0-to-1-years-040825505099</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.naukri.com/job-listings-junior-net-developer-truetech-solutions-mumbai-pune-1-to-2-years-050526021901</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.naukri.com/job-listings-java-or-net-developer-squircle-it-consulting-services-pvt-ltd-bengaluru-1-to-6-years-140126503565</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.naukri.com/job-listings-net-developer-informist-media-private-limited-mumbai-3-to-6-years-140526933435</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Need to answer questions</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Manual input required</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Need manual answers for questions: Enter mobile number</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.naukri.com/job-listings-senior-net-developer-technical-development-lead-dogma-group-kolkata-mumbai-new-delhi-hyderabad-pune-chennai-bengaluru-6-to-11-years-270625500169</x:t>
+  </x:si>
 </x:sst>
 </file>
 
@@ -89,7 +137,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="0" formatCode=""/>
   </x:numFmts>
-  <x:fonts count="3">
+  <x:fonts count="4">
     <x:font>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
@@ -113,8 +161,17 @@
       <x:name val="Calibri"/>
       <x:family val="2"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:u val="single"/>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color theme="10"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -124,6 +181,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF0F8FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFE0"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -146,7 +208,7 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="4">
+  <x:cellStyleXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -159,8 +221,17 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="22" fontId="1" fillId="3" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="4">
+  <x:cellXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -174,6 +245,18 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="22" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -479,10 +562,10 @@
     <x:col min="2" max="2" width="7.853482" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="9.567768" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="8.567768" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="143.139196" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="15.282054" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="8.139196" style="0" customWidth="1"/>
-    <x:col min="8" max="8" width="45.424911" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="176.424911" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24.282054" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="21.567768" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="55.710625" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:8">
@@ -771,18 +854,207 @@
         <x:v>12</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" spans="1:8" s="4" customFormat="1">
+      <x:c r="A12" s="5">
+        <x:v>46163.0844252199</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G12" s="4" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" spans="1:8">
+      <x:c r="A13" s="2">
+        <x:v>46163.0844746759</x:v>
+      </x:c>
+      <x:c r="B13" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C13" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D13" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E13" s="3" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="F13" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G13" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="H13" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" spans="1:8" s="4" customFormat="1">
+      <x:c r="A14" s="5">
+        <x:v>46163.0849738194</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G14" s="4" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" spans="1:8">
+      <x:c r="A15" s="2">
+        <x:v>46163.0850262616</x:v>
+      </x:c>
+      <x:c r="B15" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C15" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D15" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E15" s="3" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F15" s="0" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G15" s="0" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="H15" s="0" t="s">
+        <x:v>29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" spans="1:8" s="4" customFormat="1">
+      <x:c r="A16" s="5">
+        <x:v>46163.0855190741</x:v>
+      </x:c>
+      <x:c r="B16" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C16" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D16" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="F16" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G16" s="4" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H16" s="4" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" spans="1:8">
+      <x:c r="A17" s="2">
+        <x:v>46163.0855877083</x:v>
+      </x:c>
+      <x:c r="B17" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C17" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D17" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E17" s="3" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="F17" s="0" t="s">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="G17" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="H17" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" spans="1:8" s="4" customFormat="1">
+      <x:c r="A18" s="5">
+        <x:v>46163.0856853356</x:v>
+      </x:c>
+      <x:c r="B18" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C18" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D18" s="4" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E18" s="6" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="F18" s="4" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="G18" s="4" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H18" s="4" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink ref="E2" r:id="rId5"/>
-    <x:hyperlink ref="E3" r:id="rId6"/>
-    <x:hyperlink ref="E4" r:id="rId7"/>
-    <x:hyperlink ref="E5" r:id="rId8"/>
-    <x:hyperlink ref="E6" r:id="rId9"/>
-    <x:hyperlink ref="E7" r:id="rId10"/>
-    <x:hyperlink ref="E8" r:id="rId11"/>
-    <x:hyperlink ref="E9" r:id="rId12"/>
-    <x:hyperlink ref="E10" r:id="rId13"/>
-    <x:hyperlink ref="E11" r:id="rId14"/>
+    <x:hyperlink ref="E2" r:id="rId15"/>
+    <x:hyperlink ref="E3" r:id="rId17"/>
+    <x:hyperlink ref="E4" r:id="rId18"/>
+    <x:hyperlink ref="E5" r:id="rId19"/>
+    <x:hyperlink ref="E6" r:id="rId20"/>
+    <x:hyperlink ref="E7" r:id="rId21"/>
+    <x:hyperlink ref="E8" r:id="rId22"/>
+    <x:hyperlink ref="E9" r:id="rId23"/>
+    <x:hyperlink ref="E10" r:id="rId24"/>
+    <x:hyperlink ref="E11" r:id="rId25"/>
+    <x:hyperlink ref="E12" r:id="rId26"/>
+    <x:hyperlink ref="E13" r:id="rId27"/>
+    <x:hyperlink ref="E14" r:id="rId28"/>
+    <x:hyperlink ref="E15" r:id="rId29"/>
+    <x:hyperlink ref="E16" r:id="rId30"/>
+    <x:hyperlink ref="E17" r:id="rId31"/>
+    <x:hyperlink ref="E18" r:id="rId32"/>
   </x:hyperlinks>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>